<commit_message>
Flesh out more of the PIPs around the left side iO Banks + Add IOPad class and functionality to prepare for IOBank GUIs, instead of pure inptus
</commit_message>
<xml_diff>
--- a/bitstream/XC2064.xlsx
+++ b/bitstream/XC2064.xlsx
@@ -5855,22 +5855,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="X7" s="1" t="inlineStr">
         <is>
           <t>CLB HH Set A/F</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="Y7" s="1" t="inlineStr">
         <is>
           <t>CLB HH Set-Enable</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="Z7" s="1" t="inlineStr">
         <is>
           <t>CLB HH Reset-Enable</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr">
+      <c r="AA7" s="1" t="inlineStr">
         <is>
           <t>CLB HH Reset D/G</t>
         </is>
@@ -5945,22 +5945,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AP7" t="inlineStr">
+      <c r="AP7" s="1" t="inlineStr">
         <is>
           <t>CLB HG Set A/F</t>
         </is>
       </c>
-      <c r="AQ7" t="inlineStr">
+      <c r="AQ7" s="1" t="inlineStr">
         <is>
           <t>CLB HG Set-Enable</t>
         </is>
       </c>
-      <c r="AR7" t="inlineStr">
+      <c r="AR7" s="1" t="inlineStr">
         <is>
           <t>CLB HG Reset-Enable</t>
         </is>
       </c>
-      <c r="AS7" t="inlineStr">
+      <c r="AS7" s="1" t="inlineStr">
         <is>
           <t>CLB HG Reset D/G</t>
         </is>
@@ -6045,22 +6045,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BJ7" t="inlineStr">
+      <c r="BJ7" s="1" t="inlineStr">
         <is>
           <t>CLB HF Set A/F</t>
         </is>
       </c>
-      <c r="BK7" t="inlineStr">
+      <c r="BK7" s="1" t="inlineStr">
         <is>
           <t>CLB HF Set-Enable</t>
         </is>
       </c>
-      <c r="BL7" t="inlineStr">
+      <c r="BL7" s="1" t="inlineStr">
         <is>
           <t>CLB HF Reset-Enable</t>
         </is>
       </c>
-      <c r="BM7" t="inlineStr">
+      <c r="BM7" s="1" t="inlineStr">
         <is>
           <t>CLB HF Reset D/G</t>
         </is>
@@ -6135,22 +6135,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CB7" t="inlineStr">
+      <c r="CB7" s="1" t="inlineStr">
         <is>
           <t>CLB HE Set A/F</t>
         </is>
       </c>
-      <c r="CC7" t="inlineStr">
+      <c r="CC7" s="1" t="inlineStr">
         <is>
           <t>CLB HE Set-Enable</t>
         </is>
       </c>
-      <c r="CD7" t="inlineStr">
+      <c r="CD7" s="1" t="inlineStr">
         <is>
           <t>CLB HE Reset-Enable</t>
         </is>
       </c>
-      <c r="CE7" t="inlineStr">
+      <c r="CE7" s="1" t="inlineStr">
         <is>
           <t>CLB HE Reset D/G</t>
         </is>
@@ -6225,22 +6225,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CT7" t="inlineStr">
+      <c r="CT7" s="1" t="inlineStr">
         <is>
           <t>CLB HD Set A/F</t>
         </is>
       </c>
-      <c r="CU7" t="inlineStr">
+      <c r="CU7" s="1" t="inlineStr">
         <is>
           <t>CLB HD Set-Enable</t>
         </is>
       </c>
-      <c r="CV7" t="inlineStr">
+      <c r="CV7" s="1" t="inlineStr">
         <is>
           <t>CLB HD Reset-Enable</t>
         </is>
       </c>
-      <c r="CW7" t="inlineStr">
+      <c r="CW7" s="1" t="inlineStr">
         <is>
           <t>CLB HD Reset D/G</t>
         </is>
@@ -6325,22 +6325,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DN7" t="inlineStr">
+      <c r="DN7" s="1" t="inlineStr">
         <is>
           <t>CLB HC Set A/F</t>
         </is>
       </c>
-      <c r="DO7" t="inlineStr">
+      <c r="DO7" s="1" t="inlineStr">
         <is>
           <t>CLB HC Set-Enable</t>
         </is>
       </c>
-      <c r="DP7" t="inlineStr">
+      <c r="DP7" s="1" t="inlineStr">
         <is>
           <t>CLB HC Reset-Enable</t>
         </is>
       </c>
-      <c r="DQ7" t="inlineStr">
+      <c r="DQ7" s="1" t="inlineStr">
         <is>
           <t>CLB HC Reset D/G</t>
         </is>
@@ -6415,22 +6415,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EF7" t="inlineStr">
+      <c r="EF7" s="1" t="inlineStr">
         <is>
           <t>CLB HB Set A/F</t>
         </is>
       </c>
-      <c r="EG7" t="inlineStr">
+      <c r="EG7" s="1" t="inlineStr">
         <is>
           <t>CLB HB Set-Enable</t>
         </is>
       </c>
-      <c r="EH7" t="inlineStr">
+      <c r="EH7" s="1" t="inlineStr">
         <is>
           <t>CLB HB Reset-Enable</t>
         </is>
       </c>
-      <c r="EI7" t="inlineStr">
+      <c r="EI7" s="1" t="inlineStr">
         <is>
           <t>CLB HB Reset D/G</t>
         </is>
@@ -6505,22 +6505,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EX7" t="inlineStr">
+      <c r="EX7" s="1" t="inlineStr">
         <is>
           <t>CLB HA Set A/F</t>
         </is>
       </c>
-      <c r="EY7" t="inlineStr">
+      <c r="EY7" s="1" t="inlineStr">
         <is>
           <t>CLB HA Set-Enable</t>
         </is>
       </c>
-      <c r="EZ7" t="inlineStr">
+      <c r="EZ7" s="1" t="inlineStr">
         <is>
           <t>CLB HA Reset-Enable</t>
         </is>
       </c>
-      <c r="FA7" t="inlineStr">
+      <c r="FA7" s="1" t="inlineStr">
         <is>
           <t>CLB HA Reset D/G</t>
         </is>
@@ -12271,22 +12271,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="X15" s="1" t="inlineStr">
         <is>
           <t>CLB GH Set A/F</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="Y15" s="1" t="inlineStr">
         <is>
           <t>CLB GH Set-Enable</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr">
+      <c r="Z15" s="1" t="inlineStr">
         <is>
           <t>CLB GH Reset-Enable</t>
         </is>
       </c>
-      <c r="AA15" t="inlineStr">
+      <c r="AA15" s="1" t="inlineStr">
         <is>
           <t>CLB GH Reset D/G</t>
         </is>
@@ -12361,22 +12361,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AP15" t="inlineStr">
+      <c r="AP15" s="1" t="inlineStr">
         <is>
           <t>CLB GG Set A/F</t>
         </is>
       </c>
-      <c r="AQ15" t="inlineStr">
+      <c r="AQ15" s="1" t="inlineStr">
         <is>
           <t>CLB GG Set-Enable</t>
         </is>
       </c>
-      <c r="AR15" t="inlineStr">
+      <c r="AR15" s="1" t="inlineStr">
         <is>
           <t>CLB GG Reset-Enable</t>
         </is>
       </c>
-      <c r="AS15" t="inlineStr">
+      <c r="AS15" s="1" t="inlineStr">
         <is>
           <t>CLB GG Reset D/G</t>
         </is>
@@ -12461,22 +12461,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BJ15" t="inlineStr">
+      <c r="BJ15" s="1" t="inlineStr">
         <is>
           <t>CLB GF Set A/F</t>
         </is>
       </c>
-      <c r="BK15" t="inlineStr">
+      <c r="BK15" s="1" t="inlineStr">
         <is>
           <t>CLB GF Set-Enable</t>
         </is>
       </c>
-      <c r="BL15" t="inlineStr">
+      <c r="BL15" s="1" t="inlineStr">
         <is>
           <t>CLB GF Reset-Enable</t>
         </is>
       </c>
-      <c r="BM15" t="inlineStr">
+      <c r="BM15" s="1" t="inlineStr">
         <is>
           <t>CLB GF Reset D/G</t>
         </is>
@@ -12551,22 +12551,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CB15" t="inlineStr">
+      <c r="CB15" s="1" t="inlineStr">
         <is>
           <t>CLB GE Set A/F</t>
         </is>
       </c>
-      <c r="CC15" t="inlineStr">
+      <c r="CC15" s="1" t="inlineStr">
         <is>
           <t>CLB GE Set-Enable</t>
         </is>
       </c>
-      <c r="CD15" t="inlineStr">
+      <c r="CD15" s="1" t="inlineStr">
         <is>
           <t>CLB GE Reset-Enable</t>
         </is>
       </c>
-      <c r="CE15" t="inlineStr">
+      <c r="CE15" s="1" t="inlineStr">
         <is>
           <t>CLB GE Reset D/G</t>
         </is>
@@ -12641,22 +12641,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CT15" t="inlineStr">
+      <c r="CT15" s="1" t="inlineStr">
         <is>
           <t>CLB GD Set A/F</t>
         </is>
       </c>
-      <c r="CU15" t="inlineStr">
+      <c r="CU15" s="1" t="inlineStr">
         <is>
           <t>CLB GD Set-Enable</t>
         </is>
       </c>
-      <c r="CV15" t="inlineStr">
+      <c r="CV15" s="1" t="inlineStr">
         <is>
           <t>CLB GD Reset-Enable</t>
         </is>
       </c>
-      <c r="CW15" t="inlineStr">
+      <c r="CW15" s="1" t="inlineStr">
         <is>
           <t>CLB GD Reset D/G</t>
         </is>
@@ -12741,22 +12741,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DN15" t="inlineStr">
+      <c r="DN15" s="1" t="inlineStr">
         <is>
           <t>CLB GC Set A/F</t>
         </is>
       </c>
-      <c r="DO15" t="inlineStr">
+      <c r="DO15" s="1" t="inlineStr">
         <is>
           <t>CLB GC Set-Enable</t>
         </is>
       </c>
-      <c r="DP15" t="inlineStr">
+      <c r="DP15" s="1" t="inlineStr">
         <is>
           <t>CLB GC Reset-Enable</t>
         </is>
       </c>
-      <c r="DQ15" t="inlineStr">
+      <c r="DQ15" s="1" t="inlineStr">
         <is>
           <t>CLB GC Reset D/G</t>
         </is>
@@ -12831,22 +12831,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EF15" t="inlineStr">
+      <c r="EF15" s="1" t="inlineStr">
         <is>
           <t>CLB GB Set A/F</t>
         </is>
       </c>
-      <c r="EG15" t="inlineStr">
+      <c r="EG15" s="1" t="inlineStr">
         <is>
           <t>CLB GB Set-Enable</t>
         </is>
       </c>
-      <c r="EH15" t="inlineStr">
+      <c r="EH15" s="1" t="inlineStr">
         <is>
           <t>CLB GB Reset-Enable</t>
         </is>
       </c>
-      <c r="EI15" t="inlineStr">
+      <c r="EI15" s="1" t="inlineStr">
         <is>
           <t>CLB GB Reset D/G</t>
         </is>
@@ -12921,22 +12921,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EX15" t="inlineStr">
+      <c r="EX15" s="1" t="inlineStr">
         <is>
           <t>CLB GA Set A/F</t>
         </is>
       </c>
-      <c r="EY15" t="inlineStr">
+      <c r="EY15" s="1" t="inlineStr">
         <is>
           <t>CLB GA Set-Enable</t>
         </is>
       </c>
-      <c r="EZ15" t="inlineStr">
+      <c r="EZ15" s="1" t="inlineStr">
         <is>
           <t>CLB GA Reset-Enable</t>
         </is>
       </c>
-      <c r="FA15" t="inlineStr">
+      <c r="FA15" s="1" t="inlineStr">
         <is>
           <t>CLB GA Reset D/G</t>
         </is>
@@ -19489,22 +19489,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
+      <c r="X24" s="1" t="inlineStr">
         <is>
           <t>CLB FH Set A/F</t>
         </is>
       </c>
-      <c r="Y24" t="inlineStr">
+      <c r="Y24" s="1" t="inlineStr">
         <is>
           <t>CLB FH Set-Enable</t>
         </is>
       </c>
-      <c r="Z24" t="inlineStr">
+      <c r="Z24" s="1" t="inlineStr">
         <is>
           <t>CLB FH Reset-Enable</t>
         </is>
       </c>
-      <c r="AA24" t="inlineStr">
+      <c r="AA24" s="1" t="inlineStr">
         <is>
           <t>CLB FH Reset D/G</t>
         </is>
@@ -19579,22 +19579,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AP24" t="inlineStr">
+      <c r="AP24" s="1" t="inlineStr">
         <is>
           <t>CLB FG Set A/F</t>
         </is>
       </c>
-      <c r="AQ24" t="inlineStr">
+      <c r="AQ24" s="1" t="inlineStr">
         <is>
           <t>CLB FG Set-Enable</t>
         </is>
       </c>
-      <c r="AR24" t="inlineStr">
+      <c r="AR24" s="1" t="inlineStr">
         <is>
           <t>CLB FG Reset-Enable</t>
         </is>
       </c>
-      <c r="AS24" t="inlineStr">
+      <c r="AS24" s="1" t="inlineStr">
         <is>
           <t>CLB FG Reset D/G</t>
         </is>
@@ -19679,22 +19679,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BJ24" t="inlineStr">
+      <c r="BJ24" s="1" t="inlineStr">
         <is>
           <t>CLB FF Set A/F</t>
         </is>
       </c>
-      <c r="BK24" t="inlineStr">
+      <c r="BK24" s="1" t="inlineStr">
         <is>
           <t>CLB FF Set-Enable</t>
         </is>
       </c>
-      <c r="BL24" t="inlineStr">
+      <c r="BL24" s="1" t="inlineStr">
         <is>
           <t>CLB FF Reset-Enable</t>
         </is>
       </c>
-      <c r="BM24" t="inlineStr">
+      <c r="BM24" s="1" t="inlineStr">
         <is>
           <t>CLB FF Reset D/G</t>
         </is>
@@ -19769,22 +19769,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CB24" t="inlineStr">
+      <c r="CB24" s="1" t="inlineStr">
         <is>
           <t>CLB FE Set A/F</t>
         </is>
       </c>
-      <c r="CC24" t="inlineStr">
+      <c r="CC24" s="1" t="inlineStr">
         <is>
           <t>CLB FE Set-Enable</t>
         </is>
       </c>
-      <c r="CD24" t="inlineStr">
+      <c r="CD24" s="1" t="inlineStr">
         <is>
           <t>CLB FE Reset-Enable</t>
         </is>
       </c>
-      <c r="CE24" t="inlineStr">
+      <c r="CE24" s="1" t="inlineStr">
         <is>
           <t>CLB FE Reset D/G</t>
         </is>
@@ -19859,22 +19859,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CT24" t="inlineStr">
+      <c r="CT24" s="1" t="inlineStr">
         <is>
           <t>CLB FD Set A/F</t>
         </is>
       </c>
-      <c r="CU24" t="inlineStr">
+      <c r="CU24" s="1" t="inlineStr">
         <is>
           <t>CLB FD Set-Enable</t>
         </is>
       </c>
-      <c r="CV24" t="inlineStr">
+      <c r="CV24" s="1" t="inlineStr">
         <is>
           <t>CLB FD Reset-Enable</t>
         </is>
       </c>
-      <c r="CW24" t="inlineStr">
+      <c r="CW24" s="1" t="inlineStr">
         <is>
           <t>CLB FD Reset D/G</t>
         </is>
@@ -19959,22 +19959,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DN24" t="inlineStr">
+      <c r="DN24" s="1" t="inlineStr">
         <is>
           <t>CLB FC Set A/F</t>
         </is>
       </c>
-      <c r="DO24" t="inlineStr">
+      <c r="DO24" s="1" t="inlineStr">
         <is>
           <t>CLB FC Set-Enable</t>
         </is>
       </c>
-      <c r="DP24" t="inlineStr">
+      <c r="DP24" s="1" t="inlineStr">
         <is>
           <t>CLB FC Reset-Enable</t>
         </is>
       </c>
-      <c r="DQ24" t="inlineStr">
+      <c r="DQ24" s="1" t="inlineStr">
         <is>
           <t>CLB FC Reset D/G</t>
         </is>
@@ -20049,22 +20049,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EF24" t="inlineStr">
+      <c r="EF24" s="1" t="inlineStr">
         <is>
           <t>CLB FB Set A/F</t>
         </is>
       </c>
-      <c r="EG24" t="inlineStr">
+      <c r="EG24" s="1" t="inlineStr">
         <is>
           <t>CLB FB Set-Enable</t>
         </is>
       </c>
-      <c r="EH24" t="inlineStr">
+      <c r="EH24" s="1" t="inlineStr">
         <is>
           <t>CLB FB Reset-Enable</t>
         </is>
       </c>
-      <c r="EI24" t="inlineStr">
+      <c r="EI24" s="1" t="inlineStr">
         <is>
           <t>CLB FB Reset D/G</t>
         </is>
@@ -20139,22 +20139,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EX24" t="inlineStr">
+      <c r="EX24" s="1" t="inlineStr">
         <is>
           <t>CLB FA Set A/F</t>
         </is>
       </c>
-      <c r="EY24" t="inlineStr">
+      <c r="EY24" s="1" t="inlineStr">
         <is>
           <t>CLB FA Set-Enable</t>
         </is>
       </c>
-      <c r="EZ24" t="inlineStr">
+      <c r="EZ24" s="1" t="inlineStr">
         <is>
           <t>CLB FA Reset-Enable</t>
         </is>
       </c>
-      <c r="FA24" t="inlineStr">
+      <c r="FA24" s="1" t="inlineStr">
         <is>
           <t>CLB FA Reset D/G</t>
         </is>
@@ -25905,22 +25905,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr">
+      <c r="X32" s="1" t="inlineStr">
         <is>
           <t>CLB EH Set A/F</t>
         </is>
       </c>
-      <c r="Y32" t="inlineStr">
+      <c r="Y32" s="1" t="inlineStr">
         <is>
           <t>CLB EH Set-Enable</t>
         </is>
       </c>
-      <c r="Z32" t="inlineStr">
+      <c r="Z32" s="1" t="inlineStr">
         <is>
           <t>CLB EH Reset-Enable</t>
         </is>
       </c>
-      <c r="AA32" t="inlineStr">
+      <c r="AA32" s="1" t="inlineStr">
         <is>
           <t>CLB EH Reset D/G</t>
         </is>
@@ -25995,22 +25995,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AP32" t="inlineStr">
+      <c r="AP32" s="1" t="inlineStr">
         <is>
           <t>CLB EG Set A/F</t>
         </is>
       </c>
-      <c r="AQ32" t="inlineStr">
+      <c r="AQ32" s="1" t="inlineStr">
         <is>
           <t>CLB EG Set-Enable</t>
         </is>
       </c>
-      <c r="AR32" t="inlineStr">
+      <c r="AR32" s="1" t="inlineStr">
         <is>
           <t>CLB EG Reset-Enable</t>
         </is>
       </c>
-      <c r="AS32" t="inlineStr">
+      <c r="AS32" s="1" t="inlineStr">
         <is>
           <t>CLB EG Reset D/G</t>
         </is>
@@ -26095,22 +26095,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BJ32" t="inlineStr">
+      <c r="BJ32" s="1" t="inlineStr">
         <is>
           <t>CLB EF Set A/F</t>
         </is>
       </c>
-      <c r="BK32" t="inlineStr">
+      <c r="BK32" s="1" t="inlineStr">
         <is>
           <t>CLB EF Set-Enable</t>
         </is>
       </c>
-      <c r="BL32" t="inlineStr">
+      <c r="BL32" s="1" t="inlineStr">
         <is>
           <t>CLB EF Reset-Enable</t>
         </is>
       </c>
-      <c r="BM32" t="inlineStr">
+      <c r="BM32" s="1" t="inlineStr">
         <is>
           <t>CLB EF Reset D/G</t>
         </is>
@@ -26185,22 +26185,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CB32" t="inlineStr">
+      <c r="CB32" s="1" t="inlineStr">
         <is>
           <t>CLB EE Set A/F</t>
         </is>
       </c>
-      <c r="CC32" t="inlineStr">
+      <c r="CC32" s="1" t="inlineStr">
         <is>
           <t>CLB EE Set-Enable</t>
         </is>
       </c>
-      <c r="CD32" t="inlineStr">
+      <c r="CD32" s="1" t="inlineStr">
         <is>
           <t>CLB EE Reset-Enable</t>
         </is>
       </c>
-      <c r="CE32" t="inlineStr">
+      <c r="CE32" s="1" t="inlineStr">
         <is>
           <t>CLB EE Reset D/G</t>
         </is>
@@ -26275,22 +26275,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CT32" t="inlineStr">
+      <c r="CT32" s="1" t="inlineStr">
         <is>
           <t>CLB ED Set A/F</t>
         </is>
       </c>
-      <c r="CU32" t="inlineStr">
+      <c r="CU32" s="1" t="inlineStr">
         <is>
           <t>CLB ED Set-Enable</t>
         </is>
       </c>
-      <c r="CV32" t="inlineStr">
+      <c r="CV32" s="1" t="inlineStr">
         <is>
           <t>CLB ED Reset-Enable</t>
         </is>
       </c>
-      <c r="CW32" t="inlineStr">
+      <c r="CW32" s="1" t="inlineStr">
         <is>
           <t>CLB ED Reset D/G</t>
         </is>
@@ -26375,22 +26375,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DN32" t="inlineStr">
+      <c r="DN32" s="1" t="inlineStr">
         <is>
           <t>CLB EC Set A/F</t>
         </is>
       </c>
-      <c r="DO32" t="inlineStr">
+      <c r="DO32" s="1" t="inlineStr">
         <is>
           <t>CLB EC Set-Enable</t>
         </is>
       </c>
-      <c r="DP32" t="inlineStr">
+      <c r="DP32" s="1" t="inlineStr">
         <is>
           <t>CLB EC Reset-Enable</t>
         </is>
       </c>
-      <c r="DQ32" t="inlineStr">
+      <c r="DQ32" s="1" t="inlineStr">
         <is>
           <t>CLB EC Reset D/G</t>
         </is>
@@ -26465,22 +26465,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EF32" t="inlineStr">
+      <c r="EF32" s="1" t="inlineStr">
         <is>
           <t>CLB EB Set A/F</t>
         </is>
       </c>
-      <c r="EG32" t="inlineStr">
+      <c r="EG32" s="1" t="inlineStr">
         <is>
           <t>CLB EB Set-Enable</t>
         </is>
       </c>
-      <c r="EH32" t="inlineStr">
+      <c r="EH32" s="1" t="inlineStr">
         <is>
           <t>CLB EB Reset-Enable</t>
         </is>
       </c>
-      <c r="EI32" t="inlineStr">
+      <c r="EI32" s="1" t="inlineStr">
         <is>
           <t>CLB EB Reset D/G</t>
         </is>
@@ -26555,22 +26555,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EX32" t="inlineStr">
+      <c r="EX32" s="1" t="inlineStr">
         <is>
           <t>CLB EA Set A/F</t>
         </is>
       </c>
-      <c r="EY32" t="inlineStr">
+      <c r="EY32" s="1" t="inlineStr">
         <is>
           <t>CLB EA Set-Enable</t>
         </is>
       </c>
-      <c r="EZ32" t="inlineStr">
+      <c r="EZ32" s="1" t="inlineStr">
         <is>
           <t>CLB EA Reset-Enable</t>
         </is>
       </c>
-      <c r="FA32" t="inlineStr">
+      <c r="FA32" s="1" t="inlineStr">
         <is>
           <t>CLB EA Reset D/G</t>
         </is>
@@ -32321,22 +32321,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr">
+      <c r="X40" s="1" t="inlineStr">
         <is>
           <t>CLB DH Set A/F</t>
         </is>
       </c>
-      <c r="Y40" t="inlineStr">
+      <c r="Y40" s="1" t="inlineStr">
         <is>
           <t>CLB DH Set-Enable</t>
         </is>
       </c>
-      <c r="Z40" t="inlineStr">
+      <c r="Z40" s="1" t="inlineStr">
         <is>
           <t>CLB DH Reset-Enable</t>
         </is>
       </c>
-      <c r="AA40" t="inlineStr">
+      <c r="AA40" s="1" t="inlineStr">
         <is>
           <t>CLB DH Reset D/G</t>
         </is>
@@ -32411,22 +32411,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AP40" t="inlineStr">
+      <c r="AP40" s="1" t="inlineStr">
         <is>
           <t>CLB DG Set A/F</t>
         </is>
       </c>
-      <c r="AQ40" t="inlineStr">
+      <c r="AQ40" s="1" t="inlineStr">
         <is>
           <t>CLB DG Set-Enable</t>
         </is>
       </c>
-      <c r="AR40" t="inlineStr">
+      <c r="AR40" s="1" t="inlineStr">
         <is>
           <t>CLB DG Reset-Enable</t>
         </is>
       </c>
-      <c r="AS40" t="inlineStr">
+      <c r="AS40" s="1" t="inlineStr">
         <is>
           <t>CLB DG Reset D/G</t>
         </is>
@@ -32511,22 +32511,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BJ40" t="inlineStr">
+      <c r="BJ40" s="1" t="inlineStr">
         <is>
           <t>CLB DF Set A/F</t>
         </is>
       </c>
-      <c r="BK40" t="inlineStr">
+      <c r="BK40" s="1" t="inlineStr">
         <is>
           <t>CLB DF Set-Enable</t>
         </is>
       </c>
-      <c r="BL40" t="inlineStr">
+      <c r="BL40" s="1" t="inlineStr">
         <is>
           <t>CLB DF Reset-Enable</t>
         </is>
       </c>
-      <c r="BM40" t="inlineStr">
+      <c r="BM40" s="1" t="inlineStr">
         <is>
           <t>CLB DF Reset D/G</t>
         </is>
@@ -32601,22 +32601,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CB40" t="inlineStr">
+      <c r="CB40" s="1" t="inlineStr">
         <is>
           <t>CLB DE Set A/F</t>
         </is>
       </c>
-      <c r="CC40" t="inlineStr">
+      <c r="CC40" s="1" t="inlineStr">
         <is>
           <t>CLB DE Set-Enable</t>
         </is>
       </c>
-      <c r="CD40" t="inlineStr">
+      <c r="CD40" s="1" t="inlineStr">
         <is>
           <t>CLB DE Reset-Enable</t>
         </is>
       </c>
-      <c r="CE40" t="inlineStr">
+      <c r="CE40" s="1" t="inlineStr">
         <is>
           <t>CLB DE Reset D/G</t>
         </is>
@@ -32691,22 +32691,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CT40" t="inlineStr">
+      <c r="CT40" s="1" t="inlineStr">
         <is>
           <t>CLB DD Set A/F</t>
         </is>
       </c>
-      <c r="CU40" t="inlineStr">
+      <c r="CU40" s="1" t="inlineStr">
         <is>
           <t>CLB DD Set-Enable</t>
         </is>
       </c>
-      <c r="CV40" t="inlineStr">
+      <c r="CV40" s="1" t="inlineStr">
         <is>
           <t>CLB DD Reset-Enable</t>
         </is>
       </c>
-      <c r="CW40" t="inlineStr">
+      <c r="CW40" s="1" t="inlineStr">
         <is>
           <t>CLB DD Reset D/G</t>
         </is>
@@ -32791,22 +32791,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DN40" t="inlineStr">
+      <c r="DN40" s="1" t="inlineStr">
         <is>
           <t>CLB DC Set A/F</t>
         </is>
       </c>
-      <c r="DO40" t="inlineStr">
+      <c r="DO40" s="1" t="inlineStr">
         <is>
           <t>CLB DC Set-Enable</t>
         </is>
       </c>
-      <c r="DP40" t="inlineStr">
+      <c r="DP40" s="1" t="inlineStr">
         <is>
           <t>CLB DC Reset-Enable</t>
         </is>
       </c>
-      <c r="DQ40" t="inlineStr">
+      <c r="DQ40" s="1" t="inlineStr">
         <is>
           <t>CLB DC Reset D/G</t>
         </is>
@@ -32881,22 +32881,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EF40" t="inlineStr">
+      <c r="EF40" s="1" t="inlineStr">
         <is>
           <t>CLB DB Set A/F</t>
         </is>
       </c>
-      <c r="EG40" t="inlineStr">
+      <c r="EG40" s="1" t="inlineStr">
         <is>
           <t>CLB DB Set-Enable</t>
         </is>
       </c>
-      <c r="EH40" t="inlineStr">
+      <c r="EH40" s="1" t="inlineStr">
         <is>
           <t>CLB DB Reset-Enable</t>
         </is>
       </c>
-      <c r="EI40" t="inlineStr">
+      <c r="EI40" s="1" t="inlineStr">
         <is>
           <t>CLB DB Reset D/G</t>
         </is>
@@ -32971,22 +32971,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EX40" t="inlineStr">
+      <c r="EX40" s="1" t="inlineStr">
         <is>
           <t>CLB DA Set A/F</t>
         </is>
       </c>
-      <c r="EY40" t="inlineStr">
+      <c r="EY40" s="1" t="inlineStr">
         <is>
           <t>CLB DA Set-Enable</t>
         </is>
       </c>
-      <c r="EZ40" t="inlineStr">
+      <c r="EZ40" s="1" t="inlineStr">
         <is>
           <t>CLB DA Reset-Enable</t>
         </is>
       </c>
-      <c r="FA40" t="inlineStr">
+      <c r="FA40" s="1" t="inlineStr">
         <is>
           <t>CLB DA Reset D/G</t>
         </is>
@@ -39539,22 +39539,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr">
+      <c r="X49" s="1" t="inlineStr">
         <is>
           <t>CLB CH Set A/F</t>
         </is>
       </c>
-      <c r="Y49" t="inlineStr">
+      <c r="Y49" s="1" t="inlineStr">
         <is>
           <t>CLB CH Set-Enable</t>
         </is>
       </c>
-      <c r="Z49" t="inlineStr">
+      <c r="Z49" s="1" t="inlineStr">
         <is>
           <t>CLB CH Reset-Enable</t>
         </is>
       </c>
-      <c r="AA49" t="inlineStr">
+      <c r="AA49" s="1" t="inlineStr">
         <is>
           <t>CLB CH Reset D/G</t>
         </is>
@@ -39629,22 +39629,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AP49" t="inlineStr">
+      <c r="AP49" s="1" t="inlineStr">
         <is>
           <t>CLB CG Set A/F</t>
         </is>
       </c>
-      <c r="AQ49" t="inlineStr">
+      <c r="AQ49" s="1" t="inlineStr">
         <is>
           <t>CLB CG Set-Enable</t>
         </is>
       </c>
-      <c r="AR49" t="inlineStr">
+      <c r="AR49" s="1" t="inlineStr">
         <is>
           <t>CLB CG Reset-Enable</t>
         </is>
       </c>
-      <c r="AS49" t="inlineStr">
+      <c r="AS49" s="1" t="inlineStr">
         <is>
           <t>CLB CG Reset D/G</t>
         </is>
@@ -39729,22 +39729,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BJ49" t="inlineStr">
+      <c r="BJ49" s="1" t="inlineStr">
         <is>
           <t>CLB CF Set A/F</t>
         </is>
       </c>
-      <c r="BK49" t="inlineStr">
+      <c r="BK49" s="1" t="inlineStr">
         <is>
           <t>CLB CF Set-Enable</t>
         </is>
       </c>
-      <c r="BL49" t="inlineStr">
+      <c r="BL49" s="1" t="inlineStr">
         <is>
           <t>CLB CF Reset-Enable</t>
         </is>
       </c>
-      <c r="BM49" t="inlineStr">
+      <c r="BM49" s="1" t="inlineStr">
         <is>
           <t>CLB CF Reset D/G</t>
         </is>
@@ -39819,22 +39819,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CB49" t="inlineStr">
+      <c r="CB49" s="1" t="inlineStr">
         <is>
           <t>CLB CE Set A/F</t>
         </is>
       </c>
-      <c r="CC49" t="inlineStr">
+      <c r="CC49" s="1" t="inlineStr">
         <is>
           <t>CLB CE Set-Enable</t>
         </is>
       </c>
-      <c r="CD49" t="inlineStr">
+      <c r="CD49" s="1" t="inlineStr">
         <is>
           <t>CLB CE Reset-Enable</t>
         </is>
       </c>
-      <c r="CE49" t="inlineStr">
+      <c r="CE49" s="1" t="inlineStr">
         <is>
           <t>CLB CE Reset D/G</t>
         </is>
@@ -39909,22 +39909,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CT49" t="inlineStr">
+      <c r="CT49" s="1" t="inlineStr">
         <is>
           <t>CLB CD Set A/F</t>
         </is>
       </c>
-      <c r="CU49" t="inlineStr">
+      <c r="CU49" s="1" t="inlineStr">
         <is>
           <t>CLB CD Set-Enable</t>
         </is>
       </c>
-      <c r="CV49" t="inlineStr">
+      <c r="CV49" s="1" t="inlineStr">
         <is>
           <t>CLB CD Reset-Enable</t>
         </is>
       </c>
-      <c r="CW49" t="inlineStr">
+      <c r="CW49" s="1" t="inlineStr">
         <is>
           <t>CLB CD Reset D/G</t>
         </is>
@@ -40009,22 +40009,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DN49" t="inlineStr">
+      <c r="DN49" s="1" t="inlineStr">
         <is>
           <t>CLB CC Set A/F</t>
         </is>
       </c>
-      <c r="DO49" t="inlineStr">
+      <c r="DO49" s="1" t="inlineStr">
         <is>
           <t>CLB CC Set-Enable</t>
         </is>
       </c>
-      <c r="DP49" t="inlineStr">
+      <c r="DP49" s="1" t="inlineStr">
         <is>
           <t>CLB CC Reset-Enable</t>
         </is>
       </c>
-      <c r="DQ49" t="inlineStr">
+      <c r="DQ49" s="1" t="inlineStr">
         <is>
           <t>CLB CC Reset D/G</t>
         </is>
@@ -40099,22 +40099,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EF49" t="inlineStr">
+      <c r="EF49" s="1" t="inlineStr">
         <is>
           <t>CLB CB Set A/F</t>
         </is>
       </c>
-      <c r="EG49" t="inlineStr">
+      <c r="EG49" s="1" t="inlineStr">
         <is>
           <t>CLB CB Set-Enable</t>
         </is>
       </c>
-      <c r="EH49" t="inlineStr">
+      <c r="EH49" s="1" t="inlineStr">
         <is>
           <t>CLB CB Reset-Enable</t>
         </is>
       </c>
-      <c r="EI49" t="inlineStr">
+      <c r="EI49" s="1" t="inlineStr">
         <is>
           <t>CLB CB Reset D/G</t>
         </is>
@@ -40189,22 +40189,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EX49" t="inlineStr">
+      <c r="EX49" s="1" t="inlineStr">
         <is>
           <t>CLB CA Set A/F</t>
         </is>
       </c>
-      <c r="EY49" t="inlineStr">
+      <c r="EY49" s="1" t="inlineStr">
         <is>
           <t>CLB CA Set-Enable</t>
         </is>
       </c>
-      <c r="EZ49" t="inlineStr">
+      <c r="EZ49" s="1" t="inlineStr">
         <is>
           <t>CLB CA Reset-Enable</t>
         </is>
       </c>
-      <c r="FA49" t="inlineStr">
+      <c r="FA49" s="1" t="inlineStr">
         <is>
           <t>CLB CA Reset D/G</t>
         </is>
@@ -45955,22 +45955,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="X57" t="inlineStr">
+      <c r="X57" s="1" t="inlineStr">
         <is>
           <t>CLB BH Set A/F</t>
         </is>
       </c>
-      <c r="Y57" t="inlineStr">
+      <c r="Y57" s="1" t="inlineStr">
         <is>
           <t>CLB BH Set-Enable</t>
         </is>
       </c>
-      <c r="Z57" t="inlineStr">
+      <c r="Z57" s="1" t="inlineStr">
         <is>
           <t>CLB BH Reset-Enable</t>
         </is>
       </c>
-      <c r="AA57" t="inlineStr">
+      <c r="AA57" s="1" t="inlineStr">
         <is>
           <t>CLB BH Reset D/G</t>
         </is>
@@ -46045,22 +46045,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AP57" t="inlineStr">
+      <c r="AP57" s="1" t="inlineStr">
         <is>
           <t>CLB BG Set A/F</t>
         </is>
       </c>
-      <c r="AQ57" t="inlineStr">
+      <c r="AQ57" s="1" t="inlineStr">
         <is>
           <t>CLB BG Set-Enable</t>
         </is>
       </c>
-      <c r="AR57" t="inlineStr">
+      <c r="AR57" s="1" t="inlineStr">
         <is>
           <t>CLB BG Reset-Enable</t>
         </is>
       </c>
-      <c r="AS57" t="inlineStr">
+      <c r="AS57" s="1" t="inlineStr">
         <is>
           <t>CLB BG Reset D/G</t>
         </is>
@@ -46145,22 +46145,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BJ57" t="inlineStr">
+      <c r="BJ57" s="1" t="inlineStr">
         <is>
           <t>CLB BF Set A/F</t>
         </is>
       </c>
-      <c r="BK57" t="inlineStr">
+      <c r="BK57" s="1" t="inlineStr">
         <is>
           <t>CLB BF Set-Enable</t>
         </is>
       </c>
-      <c r="BL57" t="inlineStr">
+      <c r="BL57" s="1" t="inlineStr">
         <is>
           <t>CLB BF Reset-Enable</t>
         </is>
       </c>
-      <c r="BM57" t="inlineStr">
+      <c r="BM57" s="1" t="inlineStr">
         <is>
           <t>CLB BF Reset D/G</t>
         </is>
@@ -46235,22 +46235,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CB57" t="inlineStr">
+      <c r="CB57" s="1" t="inlineStr">
         <is>
           <t>CLB BE Set A/F</t>
         </is>
       </c>
-      <c r="CC57" t="inlineStr">
+      <c r="CC57" s="1" t="inlineStr">
         <is>
           <t>CLB BE Set-Enable</t>
         </is>
       </c>
-      <c r="CD57" t="inlineStr">
+      <c r="CD57" s="1" t="inlineStr">
         <is>
           <t>CLB BE Reset-Enable</t>
         </is>
       </c>
-      <c r="CE57" t="inlineStr">
+      <c r="CE57" s="1" t="inlineStr">
         <is>
           <t>CLB BE Reset D/G</t>
         </is>
@@ -46325,22 +46325,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CT57" t="inlineStr">
+      <c r="CT57" s="1" t="inlineStr">
         <is>
           <t>CLB BD Set A/F</t>
         </is>
       </c>
-      <c r="CU57" t="inlineStr">
+      <c r="CU57" s="1" t="inlineStr">
         <is>
           <t>CLB BD Set-Enable</t>
         </is>
       </c>
-      <c r="CV57" t="inlineStr">
+      <c r="CV57" s="1" t="inlineStr">
         <is>
           <t>CLB BD Reset-Enable</t>
         </is>
       </c>
-      <c r="CW57" t="inlineStr">
+      <c r="CW57" s="1" t="inlineStr">
         <is>
           <t>CLB BD Reset D/G</t>
         </is>
@@ -46425,22 +46425,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DN57" t="inlineStr">
+      <c r="DN57" s="1" t="inlineStr">
         <is>
           <t>CLB BC Set A/F</t>
         </is>
       </c>
-      <c r="DO57" t="inlineStr">
+      <c r="DO57" s="1" t="inlineStr">
         <is>
           <t>CLB BC Set-Enable</t>
         </is>
       </c>
-      <c r="DP57" t="inlineStr">
+      <c r="DP57" s="1" t="inlineStr">
         <is>
           <t>CLB BC Reset-Enable</t>
         </is>
       </c>
-      <c r="DQ57" t="inlineStr">
+      <c r="DQ57" s="1" t="inlineStr">
         <is>
           <t>CLB BC Reset D/G</t>
         </is>
@@ -46515,22 +46515,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EF57" t="inlineStr">
+      <c r="EF57" s="1" t="inlineStr">
         <is>
           <t>CLB BB Set A/F</t>
         </is>
       </c>
-      <c r="EG57" t="inlineStr">
+      <c r="EG57" s="1" t="inlineStr">
         <is>
           <t>CLB BB Set-Enable</t>
         </is>
       </c>
-      <c r="EH57" t="inlineStr">
+      <c r="EH57" s="1" t="inlineStr">
         <is>
           <t>CLB BB Reset-Enable</t>
         </is>
       </c>
-      <c r="EI57" t="inlineStr">
+      <c r="EI57" s="1" t="inlineStr">
         <is>
           <t>CLB BB Reset D/G</t>
         </is>
@@ -46605,22 +46605,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EX57" t="inlineStr">
+      <c r="EX57" s="1" t="inlineStr">
         <is>
           <t>CLB BA Set A/F</t>
         </is>
       </c>
-      <c r="EY57" t="inlineStr">
+      <c r="EY57" s="1" t="inlineStr">
         <is>
           <t>CLB BA Set-Enable</t>
         </is>
       </c>
-      <c r="EZ57" t="inlineStr">
+      <c r="EZ57" s="1" t="inlineStr">
         <is>
           <t>CLB BA Reset-Enable</t>
         </is>
       </c>
-      <c r="FA57" t="inlineStr">
+      <c r="FA57" s="1" t="inlineStr">
         <is>
           <t>CLB BA Reset D/G</t>
         </is>
@@ -52371,22 +52371,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="X65" t="inlineStr">
+      <c r="X65" s="1" t="inlineStr">
         <is>
           <t>CLB AH Set A/F</t>
         </is>
       </c>
-      <c r="Y65" t="inlineStr">
+      <c r="Y65" s="1" t="inlineStr">
         <is>
           <t>CLB AH Set-Enable</t>
         </is>
       </c>
-      <c r="Z65" t="inlineStr">
+      <c r="Z65" s="1" t="inlineStr">
         <is>
           <t>CLB AH Reset-Enable</t>
         </is>
       </c>
-      <c r="AA65" t="inlineStr">
+      <c r="AA65" s="1" t="inlineStr">
         <is>
           <t>CLB AH Reset D/G</t>
         </is>
@@ -52461,22 +52461,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AP65" t="inlineStr">
+      <c r="AP65" s="1" t="inlineStr">
         <is>
           <t>CLB AG Set A/F</t>
         </is>
       </c>
-      <c r="AQ65" t="inlineStr">
+      <c r="AQ65" s="1" t="inlineStr">
         <is>
           <t>CLB AG Set-Enable</t>
         </is>
       </c>
-      <c r="AR65" t="inlineStr">
+      <c r="AR65" s="1" t="inlineStr">
         <is>
           <t>CLB AG Reset-Enable</t>
         </is>
       </c>
-      <c r="AS65" t="inlineStr">
+      <c r="AS65" s="1" t="inlineStr">
         <is>
           <t>CLB AG Reset D/G</t>
         </is>
@@ -52561,22 +52561,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BJ65" t="inlineStr">
+      <c r="BJ65" s="1" t="inlineStr">
         <is>
           <t>CLB AF Set A/F</t>
         </is>
       </c>
-      <c r="BK65" t="inlineStr">
+      <c r="BK65" s="1" t="inlineStr">
         <is>
           <t>CLB AF Set-Enable</t>
         </is>
       </c>
-      <c r="BL65" t="inlineStr">
+      <c r="BL65" s="1" t="inlineStr">
         <is>
           <t>CLB AF Reset-Enable</t>
         </is>
       </c>
-      <c r="BM65" t="inlineStr">
+      <c r="BM65" s="1" t="inlineStr">
         <is>
           <t>CLB AF Reset D/G</t>
         </is>
@@ -52651,22 +52651,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CB65" t="inlineStr">
+      <c r="CB65" s="1" t="inlineStr">
         <is>
           <t>CLB AE Set A/F</t>
         </is>
       </c>
-      <c r="CC65" t="inlineStr">
+      <c r="CC65" s="1" t="inlineStr">
         <is>
           <t>CLB AE Set-Enable</t>
         </is>
       </c>
-      <c r="CD65" t="inlineStr">
+      <c r="CD65" s="1" t="inlineStr">
         <is>
           <t>CLB AE Reset-Enable</t>
         </is>
       </c>
-      <c r="CE65" t="inlineStr">
+      <c r="CE65" s="1" t="inlineStr">
         <is>
           <t>CLB AE Reset D/G</t>
         </is>
@@ -52741,22 +52741,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CT65" t="inlineStr">
+      <c r="CT65" s="1" t="inlineStr">
         <is>
           <t>CLB AD Set A/F</t>
         </is>
       </c>
-      <c r="CU65" t="inlineStr">
+      <c r="CU65" s="1" t="inlineStr">
         <is>
           <t>CLB AD Set-Enable</t>
         </is>
       </c>
-      <c r="CV65" t="inlineStr">
+      <c r="CV65" s="1" t="inlineStr">
         <is>
           <t>CLB AD Reset-Enable</t>
         </is>
       </c>
-      <c r="CW65" t="inlineStr">
+      <c r="CW65" s="1" t="inlineStr">
         <is>
           <t>CLB AD Reset D/G</t>
         </is>
@@ -52841,22 +52841,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DN65" t="inlineStr">
+      <c r="DN65" s="1" t="inlineStr">
         <is>
           <t>CLB AC Set A/F</t>
         </is>
       </c>
-      <c r="DO65" t="inlineStr">
+      <c r="DO65" s="1" t="inlineStr">
         <is>
           <t>CLB AC Set-Enable</t>
         </is>
       </c>
-      <c r="DP65" t="inlineStr">
+      <c r="DP65" s="1" t="inlineStr">
         <is>
           <t>CLB AC Reset-Enable</t>
         </is>
       </c>
-      <c r="DQ65" t="inlineStr">
+      <c r="DQ65" s="1" t="inlineStr">
         <is>
           <t>CLB AC Reset D/G</t>
         </is>
@@ -52931,22 +52931,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EF65" t="inlineStr">
+      <c r="EF65" s="1" t="inlineStr">
         <is>
           <t>CLB AB Set A/F</t>
         </is>
       </c>
-      <c r="EG65" t="inlineStr">
+      <c r="EG65" s="1" t="inlineStr">
         <is>
           <t>CLB AB Set-Enable</t>
         </is>
       </c>
-      <c r="EH65" t="inlineStr">
+      <c r="EH65" s="1" t="inlineStr">
         <is>
           <t>CLB AB Reset-Enable</t>
         </is>
       </c>
-      <c r="EI65" t="inlineStr">
+      <c r="EI65" s="1" t="inlineStr">
         <is>
           <t>CLB AB Reset D/G</t>
         </is>
@@ -53021,22 +53021,22 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EX65" t="inlineStr">
+      <c r="EX65" s="1" t="inlineStr">
         <is>
           <t>CLB AA Set A/F</t>
         </is>
       </c>
-      <c r="EY65" t="inlineStr">
+      <c r="EY65" s="1" t="inlineStr">
         <is>
           <t>CLB AA Set-Enable</t>
         </is>
       </c>
-      <c r="EZ65" t="inlineStr">
+      <c r="EZ65" s="1" t="inlineStr">
         <is>
           <t>CLB AA Reset-Enable</t>
         </is>
       </c>
-      <c r="FA65" t="inlineStr">
+      <c r="FA65" s="1" t="inlineStr">
         <is>
           <t>CLB AA Reset D/G</t>
         </is>

</xml_diff>